<commit_message>
updated the crp tables - with hamming distance calculations
</commit_message>
<xml_diff>
--- a/project3_part1/tb/crp_results/crp_tables_for_report.xlsx
+++ b/project3_part1/tb/crp_results/crp_tables_for_report.xlsx
@@ -8,9 +8,12 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CRP Tables" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Single_Chip_HD" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Area" localSheetId="0">'CRP Tables'!$A$1:$B$303</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Single_Chip_HD'!$A$5:$I$21</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="1">'Single_Chip_HD'!$A$1:$I$23</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -18,8 +21,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
-  <fonts count="3">
+  <numFmts count="2">
+    <numFmt numFmtId="164" formatCode="0.0000"/>
+    <numFmt numFmtId="165" formatCode="0.0000&quot;%&quot;"/>
+  </numFmts>
+  <fonts count="6">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -37,8 +43,24 @@
       <name val="Consolas"/>
       <sz val="10"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="0017365D"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="0017365D"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="0017365D"/>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="4">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -53,6 +75,21 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00EDF1F5"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00EAF1F8"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E2F0D9"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F0F3F6"/>
       </patternFill>
     </fill>
   </fills>
@@ -115,7 +152,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -128,6 +165,36 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="49" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -3931,4 +3998,628 @@
   <pageMargins left="0.3" right="0.3" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" paperSize="9" fitToHeight="0" fitToWidth="1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A1:I23"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="17" customWidth="1" min="5" max="5"/>
+    <col width="17" customWidth="1" min="6" max="6"/>
+    <col width="20" customWidth="1" min="7" max="7"/>
+    <col width="23" customWidth="1" min="8" max="8"/>
+    <col width="23" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="27" customHeight="1">
+      <c r="A1" s="6" t="inlineStr">
+        <is>
+          <t>Single-chip Hamming distance</t>
+        </is>
+      </c>
+      <c r="B1" s="7" t="n"/>
+      <c r="C1" s="7" t="n"/>
+      <c r="D1" s="7" t="n"/>
+      <c r="E1" s="7" t="n"/>
+      <c r="F1" s="7" t="n"/>
+      <c r="G1" s="7" t="n"/>
+      <c r="H1" s="7" t="n"/>
+      <c r="I1" s="7" t="n"/>
+    </row>
+    <row r="2" ht="30" customHeight="1">
+      <c r="A2" s="8" t="inlineStr">
+        <is>
+          <t>Different-challenge variation compares responses within one PUF. Same-challenge repeatability compares the two recorded runs of each challenge.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="24" customHeight="1">
+      <c r="B4" s="9" t="inlineStr">
+        <is>
+          <t>Different-challenge variation</t>
+        </is>
+      </c>
+      <c r="C4" s="10" t="n"/>
+      <c r="D4" s="10" t="n"/>
+      <c r="E4" s="10" t="n"/>
+      <c r="F4" s="10" t="n"/>
+      <c r="G4" s="11" t="inlineStr">
+        <is>
+          <t>Same-challenge repeatability</t>
+        </is>
+      </c>
+      <c r="H4" s="12" t="n"/>
+      <c r="I4" s="12" t="n"/>
+    </row>
+    <row r="5" ht="32" customHeight="1">
+      <c r="A5" s="13" t="inlineStr">
+        <is>
+          <t>Configuration</t>
+        </is>
+      </c>
+      <c r="B5" s="13" t="inlineStr">
+        <is>
+          <t>Challenge pairs</t>
+        </is>
+      </c>
+      <c r="C5" s="13" t="inlineStr">
+        <is>
+          <t>Mean HD (bits)</t>
+        </is>
+      </c>
+      <c r="D5" s="13" t="inlineStr">
+        <is>
+          <t>Mean HD (%)</t>
+        </is>
+      </c>
+      <c r="E5" s="13" t="inlineStr">
+        <is>
+          <t>Min HD (bits)</t>
+        </is>
+      </c>
+      <c r="F5" s="13" t="inlineStr">
+        <is>
+          <t>Max HD (bits)</t>
+        </is>
+      </c>
+      <c r="G5" s="13" t="inlineStr">
+        <is>
+          <t>Repeat comparisons</t>
+        </is>
+      </c>
+      <c r="H5" s="13" t="inlineStr">
+        <is>
+          <t>Repeat mean HD (bits)</t>
+        </is>
+      </c>
+      <c r="I5" s="13" t="inlineStr">
+        <is>
+          <t>Repeat mean HD (%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="21" customHeight="1">
+      <c r="A6" s="14" t="inlineStr">
+        <is>
+          <t>PUF_00</t>
+        </is>
+      </c>
+      <c r="B6" s="15" t="n">
+        <v>120</v>
+      </c>
+      <c r="C6" s="16" t="n">
+        <v>15.64166666666667</v>
+      </c>
+      <c r="D6" s="17" t="n">
+        <v>48.88020833333334</v>
+      </c>
+      <c r="E6" s="15" t="n">
+        <v>4</v>
+      </c>
+      <c r="F6" s="15" t="n">
+        <v>29</v>
+      </c>
+      <c r="G6" s="15" t="n">
+        <v>16</v>
+      </c>
+      <c r="H6" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="I6" s="17" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" ht="21" customHeight="1">
+      <c r="A7" s="14" t="inlineStr">
+        <is>
+          <t>PUF_01</t>
+        </is>
+      </c>
+      <c r="B7" s="15" t="n">
+        <v>120</v>
+      </c>
+      <c r="C7" s="16" t="n">
+        <v>15.74166666666667</v>
+      </c>
+      <c r="D7" s="17" t="n">
+        <v>49.19270833333334</v>
+      </c>
+      <c r="E7" s="15" t="n">
+        <v>6</v>
+      </c>
+      <c r="F7" s="15" t="n">
+        <v>28</v>
+      </c>
+      <c r="G7" s="15" t="n">
+        <v>16</v>
+      </c>
+      <c r="H7" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="I7" s="17" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" ht="21" customHeight="1">
+      <c r="A8" s="14" t="inlineStr">
+        <is>
+          <t>PUF_02</t>
+        </is>
+      </c>
+      <c r="B8" s="15" t="n">
+        <v>120</v>
+      </c>
+      <c r="C8" s="16" t="n">
+        <v>15.71666666666667</v>
+      </c>
+      <c r="D8" s="17" t="n">
+        <v>49.11458333333334</v>
+      </c>
+      <c r="E8" s="15" t="n">
+        <v>4</v>
+      </c>
+      <c r="F8" s="15" t="n">
+        <v>29</v>
+      </c>
+      <c r="G8" s="15" t="n">
+        <v>16</v>
+      </c>
+      <c r="H8" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="I8" s="17" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" ht="21" customHeight="1">
+      <c r="A9" s="14" t="inlineStr">
+        <is>
+          <t>PUF_03</t>
+        </is>
+      </c>
+      <c r="B9" s="15" t="n">
+        <v>120</v>
+      </c>
+      <c r="C9" s="16" t="n">
+        <v>15.91666666666667</v>
+      </c>
+      <c r="D9" s="17" t="n">
+        <v>49.73958333333333</v>
+      </c>
+      <c r="E9" s="15" t="n">
+        <v>5</v>
+      </c>
+      <c r="F9" s="15" t="n">
+        <v>28</v>
+      </c>
+      <c r="G9" s="15" t="n">
+        <v>16</v>
+      </c>
+      <c r="H9" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="I9" s="17" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" ht="21" customHeight="1">
+      <c r="A10" s="14" t="inlineStr">
+        <is>
+          <t>PUF_04</t>
+        </is>
+      </c>
+      <c r="B10" s="15" t="n">
+        <v>120</v>
+      </c>
+      <c r="C10" s="16" t="n">
+        <v>15.64166666666667</v>
+      </c>
+      <c r="D10" s="17" t="n">
+        <v>48.88020833333334</v>
+      </c>
+      <c r="E10" s="15" t="n">
+        <v>4</v>
+      </c>
+      <c r="F10" s="15" t="n">
+        <v>28</v>
+      </c>
+      <c r="G10" s="15" t="n">
+        <v>16</v>
+      </c>
+      <c r="H10" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="I10" s="17" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" ht="21" customHeight="1">
+      <c r="A11" s="14" t="inlineStr">
+        <is>
+          <t>PUF_05</t>
+        </is>
+      </c>
+      <c r="B11" s="15" t="n">
+        <v>120</v>
+      </c>
+      <c r="C11" s="16" t="n">
+        <v>14.98333333333333</v>
+      </c>
+      <c r="D11" s="17" t="n">
+        <v>46.82291666666666</v>
+      </c>
+      <c r="E11" s="15" t="n">
+        <v>5</v>
+      </c>
+      <c r="F11" s="15" t="n">
+        <v>27</v>
+      </c>
+      <c r="G11" s="15" t="n">
+        <v>16</v>
+      </c>
+      <c r="H11" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="I11" s="17" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" ht="21" customHeight="1">
+      <c r="A12" s="14" t="inlineStr">
+        <is>
+          <t>PUF_06</t>
+        </is>
+      </c>
+      <c r="B12" s="15" t="n">
+        <v>120</v>
+      </c>
+      <c r="C12" s="16" t="n">
+        <v>15.40833333333333</v>
+      </c>
+      <c r="D12" s="17" t="n">
+        <v>48.15104166666666</v>
+      </c>
+      <c r="E12" s="15" t="n">
+        <v>4</v>
+      </c>
+      <c r="F12" s="15" t="n">
+        <v>29</v>
+      </c>
+      <c r="G12" s="15" t="n">
+        <v>16</v>
+      </c>
+      <c r="H12" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="I12" s="17" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" ht="21" customHeight="1">
+      <c r="A13" s="14" t="inlineStr">
+        <is>
+          <t>PUF_07</t>
+        </is>
+      </c>
+      <c r="B13" s="15" t="n">
+        <v>120</v>
+      </c>
+      <c r="C13" s="16" t="n">
+        <v>15.68333333333333</v>
+      </c>
+      <c r="D13" s="17" t="n">
+        <v>49.01041666666666</v>
+      </c>
+      <c r="E13" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="F13" s="15" t="n">
+        <v>29</v>
+      </c>
+      <c r="G13" s="15" t="n">
+        <v>16</v>
+      </c>
+      <c r="H13" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="I13" s="17" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" ht="21" customHeight="1">
+      <c r="A14" s="14" t="inlineStr">
+        <is>
+          <t>PUF_08</t>
+        </is>
+      </c>
+      <c r="B14" s="15" t="n">
+        <v>120</v>
+      </c>
+      <c r="C14" s="16" t="n">
+        <v>16.36666666666667</v>
+      </c>
+      <c r="D14" s="17" t="n">
+        <v>51.14583333333334</v>
+      </c>
+      <c r="E14" s="15" t="n">
+        <v>4</v>
+      </c>
+      <c r="F14" s="15" t="n">
+        <v>30</v>
+      </c>
+      <c r="G14" s="15" t="n">
+        <v>16</v>
+      </c>
+      <c r="H14" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="I14" s="17" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" ht="21" customHeight="1">
+      <c r="A15" s="14" t="inlineStr">
+        <is>
+          <t>PUF_09</t>
+        </is>
+      </c>
+      <c r="B15" s="15" t="n">
+        <v>120</v>
+      </c>
+      <c r="C15" s="16" t="n">
+        <v>15.96666666666667</v>
+      </c>
+      <c r="D15" s="17" t="n">
+        <v>49.89583333333334</v>
+      </c>
+      <c r="E15" s="15" t="n">
+        <v>4</v>
+      </c>
+      <c r="F15" s="15" t="n">
+        <v>29</v>
+      </c>
+      <c r="G15" s="15" t="n">
+        <v>16</v>
+      </c>
+      <c r="H15" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="I15" s="17" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16" ht="21" customHeight="1">
+      <c r="A16" s="14" t="inlineStr">
+        <is>
+          <t>PUF_10</t>
+        </is>
+      </c>
+      <c r="B16" s="15" t="n">
+        <v>120</v>
+      </c>
+      <c r="C16" s="16" t="n">
+        <v>15.875</v>
+      </c>
+      <c r="D16" s="17" t="n">
+        <v>49.609375</v>
+      </c>
+      <c r="E16" s="15" t="n">
+        <v>6</v>
+      </c>
+      <c r="F16" s="15" t="n">
+        <v>30</v>
+      </c>
+      <c r="G16" s="15" t="n">
+        <v>16</v>
+      </c>
+      <c r="H16" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="I16" s="17" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17" ht="21" customHeight="1">
+      <c r="A17" s="14" t="inlineStr">
+        <is>
+          <t>PUF_11</t>
+        </is>
+      </c>
+      <c r="B17" s="15" t="n">
+        <v>120</v>
+      </c>
+      <c r="C17" s="16" t="n">
+        <v>16.23333333333333</v>
+      </c>
+      <c r="D17" s="17" t="n">
+        <v>50.72916666666667</v>
+      </c>
+      <c r="E17" s="15" t="n">
+        <v>6</v>
+      </c>
+      <c r="F17" s="15" t="n">
+        <v>29</v>
+      </c>
+      <c r="G17" s="15" t="n">
+        <v>16</v>
+      </c>
+      <c r="H17" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="I17" s="17" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18" ht="21" customHeight="1">
+      <c r="A18" s="14" t="inlineStr">
+        <is>
+          <t>PUF_12</t>
+        </is>
+      </c>
+      <c r="B18" s="15" t="n">
+        <v>120</v>
+      </c>
+      <c r="C18" s="16" t="n">
+        <v>16.175</v>
+      </c>
+      <c r="D18" s="17" t="n">
+        <v>50.546875</v>
+      </c>
+      <c r="E18" s="15" t="n">
+        <v>5</v>
+      </c>
+      <c r="F18" s="15" t="n">
+        <v>29</v>
+      </c>
+      <c r="G18" s="15" t="n">
+        <v>16</v>
+      </c>
+      <c r="H18" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="I18" s="17" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19" ht="21" customHeight="1">
+      <c r="A19" s="14" t="inlineStr">
+        <is>
+          <t>PUF_13</t>
+        </is>
+      </c>
+      <c r="B19" s="15" t="n">
+        <v>120</v>
+      </c>
+      <c r="C19" s="16" t="n">
+        <v>16.375</v>
+      </c>
+      <c r="D19" s="17" t="n">
+        <v>51.171875</v>
+      </c>
+      <c r="E19" s="15" t="n">
+        <v>6</v>
+      </c>
+      <c r="F19" s="15" t="n">
+        <v>30</v>
+      </c>
+      <c r="G19" s="15" t="n">
+        <v>16</v>
+      </c>
+      <c r="H19" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="I19" s="17" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20" ht="21" customHeight="1">
+      <c r="A20" s="14" t="inlineStr">
+        <is>
+          <t>PUF_14</t>
+        </is>
+      </c>
+      <c r="B20" s="15" t="n">
+        <v>120</v>
+      </c>
+      <c r="C20" s="16" t="n">
+        <v>15.90833333333333</v>
+      </c>
+      <c r="D20" s="17" t="n">
+        <v>49.71354166666666</v>
+      </c>
+      <c r="E20" s="15" t="n">
+        <v>4</v>
+      </c>
+      <c r="F20" s="15" t="n">
+        <v>29</v>
+      </c>
+      <c r="G20" s="15" t="n">
+        <v>16</v>
+      </c>
+      <c r="H20" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="I20" s="17" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21" ht="21" customHeight="1">
+      <c r="A21" s="14" t="inlineStr">
+        <is>
+          <t>PUF_15</t>
+        </is>
+      </c>
+      <c r="B21" s="15" t="n">
+        <v>120</v>
+      </c>
+      <c r="C21" s="16" t="n">
+        <v>16.09166666666667</v>
+      </c>
+      <c r="D21" s="17" t="n">
+        <v>50.28645833333333</v>
+      </c>
+      <c r="E21" s="15" t="n">
+        <v>4</v>
+      </c>
+      <c r="F21" s="15" t="n">
+        <v>30</v>
+      </c>
+      <c r="G21" s="15" t="n">
+        <v>16</v>
+      </c>
+      <c r="H21" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="I21" s="17" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23" ht="30" customHeight="1">
+      <c r="A23" s="8" t="inlineStr">
+        <is>
+          <t>Percentages are stored as percentage values: 50 displays as 50.0000%. Zero repeat HD means the recorded responses matched across both runs.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A5:I21"/>
+  <mergeCells count="5">
+    <mergeCell ref="B4:F4"/>
+    <mergeCell ref="A2:I2"/>
+    <mergeCell ref="A1:I1"/>
+    <mergeCell ref="A23:I23"/>
+    <mergeCell ref="G4:I4"/>
+  </mergeCells>
+  <pageMargins left="0.25" right="0.25" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" paperSize="9" fitToHeight="1" fitToWidth="1"/>
+</worksheet>
 </file>
</xml_diff>